<commit_message>
Rà soát Chương 2, Chương 3 và bài báo theo dữ liệu gốc
- Chương 2: khai thác Quy chế quản trị tài sản trí tuệ năm 2024 và Kế hoạch
  07/KH-ĐHTĐ (bản quét, đã nhận dạng chữ); sửa nhận định sai về Điều 34 Quyết
  định 213; thay các số liệu không tái lập được (28/25 bài, ba đề tài không có
  bài báo) bằng số liệu từ danh mục gốc; thêm Hình 2.16 so sánh kế hoạch và
  thực hiện 2024 - 2025; cập nhật nhật ký chuẩn hóa.
- Chương 3 và bài báo: sửa ở chế độ theo dõi thay đổi các trích dẫn pháp luật
  (Điều 135 Luật Sở hữu trí tuệ, Điều 27, 28 Luật 125/2025/QH15, Điều 86,
  Quyết định 1624/QĐ-TTg, Chỉ thị 02/CT-TTg), tên đơn vị, số liệu và các
  đoạn viện dẫn khảo sát, kết quả thí điểm không có trong dữ liệu.
- Báo cáo rà soát và script dựng lại trong scripts/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThGArqDrUUsqC1zG1BQvVL
</commit_message>
<xml_diff>
--- a/Du_lieu_bieu_do_Chuong_2.xlsx
+++ b/Du_lieu_bieu_do_Chuong_2.xlsx
@@ -23,17 +23,18 @@
     <sheet name="H2.13" sheetId="14" r:id="rId14"/>
     <sheet name="H2.14" sheetId="15" r:id="rId15"/>
     <sheet name="H2.15" sheetId="16" r:id="rId16"/>
-    <sheet name="Nhat_ky_chuan_hoa" sheetId="17" r:id="rId17"/>
-    <sheet name="DL_De_tai" sheetId="18" r:id="rId18"/>
-    <sheet name="DL_TSTT" sheetId="19" r:id="rId19"/>
-    <sheet name="DL_Tieu_chi" sheetId="20" r:id="rId20"/>
+    <sheet name="H2.16" sheetId="17" r:id="rId17"/>
+    <sheet name="Nhat_ky_chuan_hoa" sheetId="18" r:id="rId18"/>
+    <sheet name="DL_De_tai" sheetId="19" r:id="rId19"/>
+    <sheet name="DL_TSTT" sheetId="20" r:id="rId20"/>
+    <sheet name="DL_Tieu_chi" sheetId="21" r:id="rId21"/>
   </sheets>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="400">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="711" uniqueCount="458">
   <si>
     <t>DỮ LIỆU VÀ BIỂU ĐỒ CHƯƠNG 2 - THỰC TRẠNG QUẢN LÝ QUYỀN SỞ HỮU TRÍ TUỆ TẠI TRƯỜNG ĐẠI HỌC THÀNH ĐÔ</t>
   </si>
@@ -185,6 +186,15 @@
     <t>H2.15</t>
   </si>
   <si>
+    <t>Hình 2.16</t>
+  </si>
+  <si>
+    <t>Tỷ lệ thực hiện so với chỉ tiêu Kế hoạch 07/KH-ĐHTĐ, cộng dồn hai năm 2024 - 2025</t>
+  </si>
+  <si>
+    <t>H2.16</t>
+  </si>
+  <si>
     <t>Các chỉnh sửa số liệu so với bản Chương 2 trước</t>
   </si>
   <si>
@@ -629,6 +639,63 @@
     <t>Đã nộp đơn đăng ký</t>
   </si>
   <si>
+    <t>Hình 2.16. Tỷ lệ thực hiện so với chỉ tiêu Kế hoạch 07/KH-ĐHTĐ, cộng dồn hai năm 2024 - 2025</t>
+  </si>
+  <si>
+    <t>Nguồn: Nhóm nghiên cứu tính toán từ mục 2.2.4 Kế hoạch số 07/KH-ĐHTĐ ngày 01 tháng 7 năm 2024 và các danh mục thống kê của Phòng Khoa học Công nghệ. Chỉ tiêu bài báo trong nước gồm bài đăng tạp chí trong nước và tạp chí của Trường; tài sản trí tuệ tính số văn bằng được cấp; không gồm tham luận hội thảo quốc gia do danh mục không có năm.</t>
+  </si>
+  <si>
+    <t>Chỉ tiêu</t>
+  </si>
+  <si>
+    <t>Nhóm</t>
+  </si>
+  <si>
+    <t>Kế hoạch 2024 - 2025</t>
+  </si>
+  <si>
+    <t>Thực hiện 2024 - 2025</t>
+  </si>
+  <si>
+    <t>Tỷ lệ thực hiện</t>
+  </si>
+  <si>
+    <t>Bài báo tạp chí quốc tế</t>
+  </si>
+  <si>
+    <t>Công bố</t>
+  </si>
+  <si>
+    <t>Sách có chỉ số ISBN</t>
+  </si>
+  <si>
+    <t>Tham luận hội thảo cấp trường</t>
+  </si>
+  <si>
+    <t>Bài báo tạp chí trong nước, gồm tạp chí của Trường</t>
+  </si>
+  <si>
+    <t>Đề tài cấp Bộ, Nhà nước</t>
+  </si>
+  <si>
+    <t>Đề tài và học liệu</t>
+  </si>
+  <si>
+    <t>Tham luận hội thảo quốc tế</t>
+  </si>
+  <si>
+    <t>Giáo trình, tài liệu tham khảo</t>
+  </si>
+  <si>
+    <t>Công nhận sáng chế, kiểu dáng, quyền tác giả</t>
+  </si>
+  <si>
+    <t>Tài sản trí tuệ</t>
+  </si>
+  <si>
+    <t>Chuyển giao công nghệ</t>
+  </si>
+  <si>
     <t>NHẬT KÝ CHUẨN HÓA SỐ LIỆU CHƯƠNG 2</t>
   </si>
   <si>
@@ -851,6 +918,117 @@
     <t>Quy tắc tại GEMINI.md</t>
   </si>
   <si>
+    <t>Quy chế quản trị tài sản trí tuệ năm 2024</t>
+  </si>
+  <si>
+    <t>Chưa được khai thác trong Chương 2</t>
+  </si>
+  <si>
+    <t>Bổ sung vào Mục 2.2.1, 2.2.2, 2.3.1, 2.5.1, 2.5.3, Bảng 2.4 và Bảng 2.6</t>
+  </si>
+  <si>
+    <t>Tai lieu thanh do/QC SHTT ĐHTĐ.docx; bản được cung cấp chưa ghi số và ngày ban hành</t>
+  </si>
+  <si>
+    <t>Điều 34 Quyết định 213 và giải pháp hữu ích</t>
+  </si>
+  <si>
+    <t>Khẳng định Điều 34 không liệt kê giải pháp hữu ích và dùng làm một nguyên nhân</t>
+  </si>
+  <si>
+    <t>Điều 34 có liệt kê bằng độc quyền giải pháp hữu ích; sửa Bảng 2.6, Mục 2.3.1, 2.5.3 và lời bình Hình 2.14</t>
+  </si>
+  <si>
+    <t>02. QĐ 213_QĐ-ĐHTĐ, Điều 34 khoản 2</t>
+  </si>
+  <si>
+    <t>Số hiệu văn bản 213</t>
+  </si>
+  <si>
+    <t>Quyết định số 213/QĐ-ĐHTĐ năm 2021</t>
+  </si>
+  <si>
+    <t>Quy chế ban hành ngày 28/12/2021 kèm văn bản số 213/QĐ-ĐHTĐ; bản quy chế ghi là Nghị quyết, Kế hoạch 07 ghi Nghị quyết số 213/NQ-HĐT-ĐHTĐ. Đề nghị thống nhất cách gọi</t>
+  </si>
+  <si>
+    <t>Trang bìa Quy chế 213; Kế hoạch 07/KH-ĐHTĐ</t>
+  </si>
+  <si>
+    <t>Mục 2.1.5, độ phủ khai báo</t>
+  </si>
+  <si>
+    <t>Hồ sơ khai 28 bài báo; 25 trên 28 tìm thấy; độ phủ 26,2%</t>
+  </si>
+  <si>
+    <t>26 đề tài khai 32 công bố; độ phủ khoảng 29,9%; bỏ tỷ lệ 89,3% vì không tái lập được từ tài liệu gốc</t>
+  </si>
+  <si>
+    <t>Cột sản phẩm nghiệm thu, danh mục đề tài cấp cơ sở</t>
+  </si>
+  <si>
+    <t>Mục 2.5.2, ý thứ sáu</t>
+  </si>
+  <si>
+    <t>Ba đề tài ghi rõ không có bài báo như cam kết</t>
+  </si>
+  <si>
+    <t>Danh mục gốc không có ghi chú này; thay bằng: 7 đề tài chỉ có báo cáo tổng kết, 5 trong số đó xếp loại Tốt</t>
+  </si>
+  <si>
+    <t>Danh mục đề tài cấp cơ sở</t>
+  </si>
+  <si>
+    <t>Mục 2.2.3, lệ phí đăng ký</t>
+  </si>
+  <si>
+    <t>Chỉ nêu không có dòng chi</t>
+  </si>
+  <si>
+    <t>Bổ sung: Điều 35 giao Phòng KHCN nộp lệ phí nhưng Điều 38 không có mục chi tương ứng</t>
+  </si>
+  <si>
+    <t>Quyết định 213, Điều 35, 38</t>
+  </si>
+  <si>
+    <t>Kế hoạch 07/KH-ĐHTĐ ngày 01/7/2024</t>
+  </si>
+  <si>
+    <t>Chưa sử dụng; tệp là bản quét</t>
+  </si>
+  <si>
+    <t>Nhận dạng chữ và đối chiếu ảnh gốc: số liệu 2021 - 2023 khớp; bổ sung Hình 2.16 so sánh kế hoạch và thực hiện</t>
+  </si>
+  <si>
+    <t>Tai lieu thanh do/KH hoạt động KHCN giai đoạn 2024-2028.pdf</t>
+  </si>
+  <si>
+    <t>Tham luận hội thảo quốc tế 2022 - 2023</t>
+  </si>
+  <si>
+    <t>Danh mục theo ngày tổ chức: 2 và 3; Kế hoạch 07 ghi 1 và 4. Chương 2 dùng số liệu danh mục</t>
+  </si>
+  <si>
+    <t>Danh mục tham luận quốc tế; Kế hoạch 07, Bảng 4</t>
+  </si>
+  <si>
+    <t>Kiểm chứng phép so khớp tác giả</t>
+  </si>
+  <si>
+    <t>Chưa kiểm chứng</t>
+  </si>
+  <si>
+    <t>Tái lập độc lập: 256 trên 405 bài khớp; Viện Y - Dược 55, Viện QT và CN 57, Viện NCGD và CGTT 17 bài; 89 người có bài, Gini 0,828; chênh 1 - 3 đơn vị do 5 họ tên trùng nhau. Giữ số liệu Chương 2</t>
+  </si>
+  <si>
+    <t>2026 DS.xlsx và hai danh mục bài báo</t>
+  </si>
+  <si>
+    <t>Nội dung chưa có tài liệu gốc trong thư mục</t>
+  </si>
+  <si>
+    <t>Điều lệ Quỹ Ngô Xuân Độ; hợp đồng của Viện NCGD và CGTT; tư cách thành viên Mạng lưới Trung tâm Hỗ trợ công nghệ và đổi mới sáng tạo từ năm 2023; đăng ký hoạt động khoa học công nghệ của Viện; sơ đồ tổ chức ngày 16/6/2026. Giữ nguyên, cần bổ sung minh chứng</t>
+  </si>
+  <si>
     <t>Tệp Du_lieu_thong_ke_KHCN_Thanh_Do_2021_2025.xlsx</t>
   </si>
   <si>
@@ -1133,9 +1311,6 @@
     <t>KHẢ NĂNG TÍNH TOÁN BỘ TIÊU CHÍ TẠI MỤC 1.4.2</t>
   </si>
   <si>
-    <t>Nhóm</t>
-  </si>
-  <si>
     <t>Tiêu chí</t>
   </si>
   <si>
@@ -1178,13 +1353,13 @@
     <t>Mức độ chuẩn hóa biểu mẫu và quy trình phối hợp</t>
   </si>
   <si>
-    <t>Có quy trình tại Điều 35, chưa có biểu mẫu nhận diện</t>
+    <t>Có quy trình tại Điều 35 Quyết định 213 và phân công tại Điều 11 Quy chế 2024, chưa có biểu mẫu khai báo</t>
   </si>
   <si>
     <t>Số lớp tập huấn sở hữu trí tuệ</t>
   </si>
   <si>
-    <t>Không có thống kê</t>
+    <t>Kế hoạch 07/KH-ĐHTĐ chỉ thống kê lượt tập huấn chung, không tách riêng sở hữu trí tuệ</t>
   </si>
   <si>
     <t>Số đơn đăng ký sở hữu công nghiệp</t>
@@ -1239,11 +1414,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
     <numFmt numFmtId="166" formatCode="0.00"/>
     <numFmt numFmtId="167" formatCode="#,##0"/>
+    <numFmt numFmtId="168" formatCode="0%"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -1344,7 +1520,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -1377,6 +1553,9 @@
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="168" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -5037,6 +5216,438 @@
         </a:p>
       </c:txPr>
     </c:legend>
+    <c:plotVisOnly val="1"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="FFFFFF"/>
+    </a:solidFill>
+    <a:ln>
+      <a:noFill/>
+    </a:ln>
+  </c:spPr>
+  <c:printSettings>
+    <c:headerFooter/>
+    <c:pageMargins b="0.75" l="0.7" r="0.7" t="0.75" header="0.3" footer="0.3"/>
+    <c:pageSetup/>
+  </c:printSettings>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart16.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1200" b="1" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="262522"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr lang="en-US" sz="1200" b="1" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="262522"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman"/>
+              </a:rPr>
+              <a:t>Hình 2.16. Tỷ lệ thực hiện so với chỉ tiêu Kế hoạch 07/KH-ĐHTĐ, cộng dồn hai năm 2024 - 2025</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:layout/>
+    </c:title>
+    <c:plotArea>
+      <c:layout/>
+      <c:barChart>
+        <c:barDir val="bar"/>
+        <c:grouping val="clustered"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'H2.16'!$E$4</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Tỷ lệ thực hiện</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="2A78D6"/>
+            </a:solidFill>
+            <a:ln w="9525">
+              <a:solidFill>
+                <a:srgbClr val="FFFFFF"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+          <c:dPt>
+            <c:idx val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="3"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="4"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="2A78D6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="7"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="1BAF7A"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="8"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="9"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="EB6834"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:srgbClr val="FFFFFF"/>
+                </a:solidFill>
+              </a:ln>
+            </c:spPr>
+          </c:dPt>
+          <c:dLbls>
+            <c:numFmt formatCode="0%" sourceLinked="0"/>
+            <c:txPr>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="900" b="0" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="262522"/>
+                    </a:solidFill>
+                    <a:latin typeface="Times New Roman"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+          </c:dLbls>
+          <c:cat>
+            <c:strRef>
+              <c:f>'H2.16'!$A$5:$A$14</c:f>
+              <c:strCache>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>Bài báo tạp chí quốc tế</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>Sách có chỉ số ISBN</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>Tham luận hội thảo cấp trường</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>Bài báo tạp chí trong nước, gồm tạp chí của Trường</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>Đề tài cấp Bộ, Nhà nước</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>Đề tài cấp cơ sở</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>Tham luận hội thảo quốc tế</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>Giáo trình, tài liệu tham khảo</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>Công nhận sáng chế, kiểu dáng, quyền tác giả</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>Chuyển giao công nghệ</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'H2.16'!$E$5:$E$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="10"/>
+                <c:pt idx="0">
+                  <c:v>2.833333333333333</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2.666666666666667</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2.233333333333333</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.645454545454546</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.071428571428571</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.9090909090909091</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.9</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.5</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="45"/>
+        <c:axId val="50160001"/>
+        <c:axId val="50160002"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="50160001"/>
+        <c:scaling>
+          <c:orientation val="maxMin"/>
+        </c:scaling>
+        <c:axPos val="l"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="8C8B86"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="262522"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50160002"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="50160002"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+          <c:min val="0"/>
+        </c:scaling>
+        <c:axPos val="t"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="6350">
+              <a:solidFill>
+                <a:srgbClr val="DEDDD8"/>
+              </a:solidFill>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:title>
+          <c:tx>
+            <c:rich>
+              <a:bodyPr/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1000" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="262522"/>
+                    </a:solidFill>
+                    <a:latin typeface="Times New Roman"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:r>
+                  <a:rPr lang="en-US" sz="1000" b="1" baseline="0">
+                    <a:solidFill>
+                      <a:srgbClr val="262522"/>
+                    </a:solidFill>
+                    <a:latin typeface="Times New Roman"/>
+                  </a:rPr>
+                  <a:t>Tỷ lệ thực hiện so với kế hoạch</a:t>
+                </a:r>
+              </a:p>
+            </c:rich>
+          </c:tx>
+          <c:layout/>
+        </c:title>
+        <c:numFmt formatCode="0%" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9525">
+            <a:solidFill>
+              <a:srgbClr val="8C8B86"/>
+            </a:solidFill>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr sz="1000" b="0" baseline="0">
+                <a:solidFill>
+                  <a:srgbClr val="262522"/>
+                </a:solidFill>
+                <a:latin typeface="Times New Roman"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:endParaRPr lang="en-US"/>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="50160001"/>
+        <c:crosses val="max"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:ln>
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
     <c:plotVisOnly val="1"/>
   </c:chart>
   <c:spPr>
@@ -9624,6 +10235,41 @@
       <xdr:colOff>314325</xdr:colOff>
       <xdr:row>33</xdr:row>
       <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame macro="">
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="2" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="0" y="0"/>
+        <a:ext cx="0" cy="0"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
+<file path=xl/drawings/drawing16.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>15</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>390525</xdr:colOff>
+      <xdr:row>51</xdr:row>
+      <xdr:rowOff>123825</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -10210,7 +10856,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C24"/>
+  <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10.7109375" customWidth="1"/>
@@ -10404,36 +11050,47 @@
         <v>49</v>
       </c>
     </row>
-    <row r="21" spans="1:3">
-      <c r="B21" s="4" t="s">
+    <row r="20" spans="1:3">
+      <c r="A20" s="4" t="s">
         <v>50</v>
       </c>
-      <c r="C21" s="5" t="s">
+      <c r="B20" s="4" t="s">
         <v>51</v>
+      </c>
+      <c r="C20" s="5" t="s">
+        <v>52</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="B22" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="B23" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="B24" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>57</v>
+        <v>58</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="B25" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>60</v>
       </c>
     </row>
   </sheetData>
@@ -10453,10 +11110,11 @@
     <hyperlink ref="C17" location="'H2.13'!A1" display="H2.13"/>
     <hyperlink ref="C18" location="'H2.14'!A1" display="H2.14"/>
     <hyperlink ref="C19" location="'H2.15'!A1" display="H2.15"/>
-    <hyperlink ref="C21" location="'Nhat_ky_chuan_hoa'!A1" display="Nhat_ky_chuan_hoa"/>
-    <hyperlink ref="C22" location="'DL_De_tai'!A1" display="DL_De_tai"/>
-    <hyperlink ref="C23" location="'DL_TSTT'!A1" display="DL_TSTT"/>
-    <hyperlink ref="C24" location="'DL_Tieu_chi'!A1" display="DL_Tieu_chi"/>
+    <hyperlink ref="C20" location="'H2.16'!A1" display="H2.16"/>
+    <hyperlink ref="C22" location="'Nhat_ky_chuan_hoa'!A1" display="Nhat_ky_chuan_hoa"/>
+    <hyperlink ref="C23" location="'DL_De_tai'!A1" display="DL_De_tai"/>
+    <hyperlink ref="C24" location="'DL_TSTT'!A1" display="DL_TSTT"/>
+    <hyperlink ref="C25" location="'DL_Tieu_chi'!A1" display="DL_Tieu_chi"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -10476,12 +11134,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -10491,15 +11149,15 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="B5" s="11">
         <v>424.75</v>
@@ -10507,7 +11165,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B6" s="11">
         <v>4670</v>
@@ -10515,7 +11173,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="B7" s="11">
         <v>5000</v>
@@ -10545,12 +11203,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -10560,24 +11218,24 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B5" s="7">
         <v>0</v>
@@ -10594,7 +11252,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B6" s="7">
         <v>3</v>
@@ -10611,7 +11269,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" s="7">
         <v>7</v>
@@ -10628,7 +11286,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="7">
         <v>5</v>
@@ -10645,7 +11303,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B9" s="7">
         <v>4</v>
@@ -10684,12 +11342,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -10699,18 +11357,18 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B5" s="7">
         <v>600</v>
@@ -10721,7 +11379,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="B6" s="7">
         <v>360</v>
@@ -10732,7 +11390,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B7" s="7">
         <v>180</v>
@@ -10743,7 +11401,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="B8" s="7">
         <v>300</v>
@@ -10754,7 +11412,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="B9" s="7">
         <v>270</v>
@@ -10765,7 +11423,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="B10" s="7">
         <v>240</v>
@@ -10776,7 +11434,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="B11" s="7">
         <v>240</v>
@@ -10787,7 +11445,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="B12" s="7">
         <v>150</v>
@@ -10820,12 +11478,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -10835,21 +11493,21 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B5" s="7">
         <v>2</v>
@@ -10863,7 +11521,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="B6" s="7">
         <v>2</v>
@@ -10877,7 +11535,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="B7" s="7">
         <v>5</v>
@@ -10891,7 +11549,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B8" s="7">
         <v>0</v>
@@ -10927,12 +11585,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -10942,24 +11600,24 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B5" s="7">
         <v>1</v>
@@ -10976,7 +11634,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B6" s="7">
         <v>0</v>
@@ -10993,7 +11651,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" s="7">
         <v>2</v>
@@ -11010,7 +11668,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="7">
         <v>0</v>
@@ -11027,7 +11685,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B9" s="7">
         <v>1</v>
@@ -11044,7 +11702,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B10" s="7">
         <v>0</v>
@@ -11083,12 +11741,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -11098,15 +11756,15 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="B5" s="7">
         <v>5</v>
@@ -11114,7 +11772,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="B6" s="7">
         <v>2</v>
@@ -11122,7 +11780,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="B7" s="7">
         <v>1</v>
@@ -11130,7 +11788,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B8" s="7">
         <v>2</v>
@@ -11138,7 +11796,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B9" s="7">
         <v>1</v>
@@ -11168,12 +11826,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -11183,18 +11841,18 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B5" s="7">
         <v>38</v>
@@ -11205,7 +11863,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B6" s="7">
         <v>11</v>
@@ -11216,7 +11874,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B7" s="7">
         <v>1</v>
@@ -11237,7 +11895,231 @@
 
 <file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D22"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:F14"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="42.7109375" customWidth="1"/>
+    <col min="2" max="5" width="17.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" ht="42" customHeight="1">
+      <c r="A2" s="6" t="s">
+        <v>202</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+    </row>
+    <row r="4" spans="1:6" ht="45" customHeight="1">
+      <c r="A4" s="3" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>204</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>206</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="4" t="s">
+        <v>208</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C5" s="7">
+        <v>30</v>
+      </c>
+      <c r="D5" s="7">
+        <v>85</v>
+      </c>
+      <c r="E5" s="12">
+        <v>2.833333333333333</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C6" s="7">
+        <v>3</v>
+      </c>
+      <c r="D6" s="7">
+        <v>8</v>
+      </c>
+      <c r="E6" s="12">
+        <v>2.666666666666667</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C7" s="7">
+        <v>60</v>
+      </c>
+      <c r="D7" s="7">
+        <v>134</v>
+      </c>
+      <c r="E7" s="12">
+        <v>2.233333333333333</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C8" s="7">
+        <v>110</v>
+      </c>
+      <c r="D8" s="7">
+        <v>181</v>
+      </c>
+      <c r="E8" s="12">
+        <v>1.645454545454546</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C9" s="7">
+        <v>2</v>
+      </c>
+      <c r="D9" s="7">
+        <v>3</v>
+      </c>
+      <c r="E9" s="12">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="4" t="s">
+        <v>83</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C10" s="7">
+        <v>14</v>
+      </c>
+      <c r="D10" s="7">
+        <v>15</v>
+      </c>
+      <c r="E10" s="12">
+        <v>1.071428571428571</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="C11" s="7">
+        <v>11</v>
+      </c>
+      <c r="D11" s="7">
+        <v>10</v>
+      </c>
+      <c r="E11" s="12">
+        <v>0.9090909090909091</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="C12" s="7">
+        <v>20</v>
+      </c>
+      <c r="D12" s="7">
+        <v>18</v>
+      </c>
+      <c r="E12" s="12">
+        <v>0.9</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="C13" s="7">
+        <v>4</v>
+      </c>
+      <c r="D13" s="7">
+        <v>6</v>
+      </c>
+      <c r="E13" s="12">
+        <v>1.5</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="C14" s="7">
+        <v>1</v>
+      </c>
+      <c r="D14" s="7">
+        <v>0</v>
+      </c>
+      <c r="E14" s="12">
+        <v>0</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" fitToHeight="0" orientation="landscape"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:D32"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
@@ -11247,287 +12129,421 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>198</v>
+        <v>220</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>199</v>
+        <v>221</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>200</v>
+        <v>222</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>201</v>
+        <v>223</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>202</v>
+        <v>224</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="4" t="s">
-        <v>203</v>
+        <v>225</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>204</v>
+        <v>226</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>205</v>
+        <v>227</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
-        <v>207</v>
+        <v>229</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>208</v>
+        <v>230</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>209</v>
+        <v>231</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>210</v>
+        <v>232</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="4" t="s">
-        <v>211</v>
+        <v>233</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>212</v>
+        <v>234</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>213</v>
+        <v>235</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>214</v>
+        <v>236</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="4" t="s">
-        <v>215</v>
+        <v>237</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>216</v>
+        <v>238</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>217</v>
+        <v>239</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>218</v>
+        <v>240</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="4" t="s">
-        <v>219</v>
+        <v>241</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>220</v>
+        <v>242</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>221</v>
+        <v>243</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>222</v>
+        <v>244</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="4" t="s">
-        <v>223</v>
+        <v>245</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>224</v>
+        <v>246</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>225</v>
+        <v>247</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>226</v>
+        <v>248</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
-        <v>227</v>
+        <v>249</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>228</v>
+        <v>250</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>229</v>
+        <v>251</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>230</v>
+        <v>252</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
-        <v>231</v>
+        <v>253</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>232</v>
+        <v>254</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>233</v>
+        <v>255</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>234</v>
+        <v>256</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="4" t="s">
-        <v>235</v>
+        <v>257</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>236</v>
+        <v>258</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>237</v>
+        <v>259</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>238</v>
+        <v>260</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>239</v>
+        <v>261</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>240</v>
+        <v>262</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>241</v>
+        <v>263</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>242</v>
+        <v>264</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="4" t="s">
-        <v>243</v>
+        <v>265</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>244</v>
+        <v>266</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>245</v>
+        <v>267</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>206</v>
+        <v>228</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="4" t="s">
-        <v>246</v>
+        <v>268</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>247</v>
+        <v>269</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>248</v>
+        <v>270</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>249</v>
+        <v>271</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="4" t="s">
-        <v>250</v>
+        <v>272</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>251</v>
+        <v>273</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>252</v>
+        <v>274</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>253</v>
+        <v>275</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="4" t="s">
-        <v>254</v>
+        <v>276</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>255</v>
+        <v>277</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="4" t="s">
-        <v>256</v>
+        <v>278</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>257</v>
+        <v>279</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>258</v>
+        <v>280</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>259</v>
+        <v>281</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="4" t="s">
-        <v>260</v>
+        <v>282</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>261</v>
+        <v>283</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>262</v>
+        <v>284</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>263</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="4" t="s">
-        <v>264</v>
+        <v>286</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>265</v>
+        <v>287</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>266</v>
+        <v>288</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>267</v>
+        <v>289</v>
       </c>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="4" t="s">
-        <v>268</v>
+        <v>290</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>269</v>
+        <v>291</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>270</v>
+        <v>292</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>271</v>
+        <v>293</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="4" t="s">
-        <v>272</v>
+        <v>294</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>273</v>
+        <v>295</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>274</v>
+        <v>296</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>275</v>
+        <v>297</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4">
+      <c r="A23" s="4" t="s">
+        <v>298</v>
+      </c>
+      <c r="B23" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="C23" s="4" t="s">
+        <v>300</v>
+      </c>
+      <c r="D23" s="4" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4">
+      <c r="A24" s="4" t="s">
+        <v>302</v>
+      </c>
+      <c r="B24" s="4" t="s">
+        <v>303</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>304</v>
+      </c>
+      <c r="D24" s="4" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4">
+      <c r="A25" s="4" t="s">
+        <v>306</v>
+      </c>
+      <c r="B25" s="4" t="s">
+        <v>307</v>
+      </c>
+      <c r="C25" s="4" t="s">
+        <v>308</v>
+      </c>
+      <c r="D25" s="4" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4">
+      <c r="A26" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B26" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>312</v>
+      </c>
+      <c r="D26" s="4" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4">
+      <c r="A27" s="4" t="s">
+        <v>314</v>
+      </c>
+      <c r="B27" s="4" t="s">
+        <v>315</v>
+      </c>
+      <c r="C27" s="4" t="s">
+        <v>316</v>
+      </c>
+      <c r="D27" s="4" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4">
+      <c r="A28" s="4" t="s">
+        <v>318</v>
+      </c>
+      <c r="B28" s="4" t="s">
+        <v>319</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>320</v>
+      </c>
+      <c r="D28" s="4" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4">
+      <c r="A29" s="4" t="s">
+        <v>322</v>
+      </c>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4" t="s">
+        <v>323</v>
+      </c>
+      <c r="D29" s="4" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4">
+      <c r="A30" s="4" t="s">
+        <v>325</v>
+      </c>
+      <c r="B30" s="4" t="s">
+        <v>326</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>327</v>
+      </c>
+      <c r="D30" s="4" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4">
+      <c r="A31" s="4" t="s">
+        <v>329</v>
+      </c>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4" t="s">
+        <v>330</v>
+      </c>
+      <c r="D31" s="4"/>
+    </row>
+    <row r="32" spans="1:4">
+      <c r="A32" s="4" t="s">
+        <v>331</v>
+      </c>
+      <c r="B32" s="4" t="s">
+        <v>332</v>
+      </c>
+      <c r="C32" s="4" t="s">
+        <v>333</v>
+      </c>
+      <c r="D32" s="4" t="s">
+        <v>334</v>
       </c>
     </row>
   </sheetData>
@@ -11535,7 +12551,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:I44"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -11548,53 +12564,53 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>276</v>
+        <v>335</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
-        <v>277</v>
+        <v>336</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>278</v>
+        <v>337</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>279</v>
+        <v>338</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>280</v>
+        <v>339</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>281</v>
+        <v>340</v>
       </c>
       <c r="G3" s="3" t="s">
-        <v>282</v>
+        <v>341</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>283</v>
+        <v>342</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="4" t="s">
-        <v>284</v>
+        <v>343</v>
       </c>
       <c r="B4" s="4">
         <v>2021</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F4" s="10">
         <v>0</v>
@@ -11605,19 +12621,19 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="4" t="s">
-        <v>287</v>
+        <v>346</v>
       </c>
       <c r="B5" s="4">
         <v>2021</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F5" s="10">
         <v>0</v>
@@ -11628,19 +12644,19 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="4" t="s">
-        <v>288</v>
+        <v>347</v>
       </c>
       <c r="B6" s="4">
         <v>2021</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F6" s="10">
         <v>0</v>
@@ -11651,19 +12667,19 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>290</v>
+        <v>349</v>
       </c>
       <c r="B7" s="4">
         <v>2021</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F7" s="10">
         <v>0</v>
@@ -11674,19 +12690,19 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4" t="s">
-        <v>291</v>
+        <v>350</v>
       </c>
       <c r="B8" s="4">
         <v>2021</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F8" s="10">
         <v>0</v>
@@ -11697,19 +12713,19 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="4" t="s">
-        <v>292</v>
+        <v>351</v>
       </c>
       <c r="B9" s="4">
         <v>2021</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F9" s="10">
         <v>0</v>
@@ -11720,19 +12736,19 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="4" t="s">
-        <v>293</v>
+        <v>352</v>
       </c>
       <c r="B10" s="4">
         <v>2022</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>294</v>
+        <v>353</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F10" s="10">
         <v>0</v>
@@ -11743,19 +12759,19 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="4" t="s">
-        <v>295</v>
+        <v>354</v>
       </c>
       <c r="B11" s="4">
         <v>2022</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F11" s="10">
         <v>0</v>
@@ -11766,19 +12782,19 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="4" t="s">
-        <v>296</v>
+        <v>355</v>
       </c>
       <c r="B12" s="4">
         <v>2022</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F12" s="10">
         <v>0</v>
@@ -11789,19 +12805,19 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="4" t="s">
-        <v>297</v>
+        <v>356</v>
       </c>
       <c r="B13" s="4">
         <v>2022</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F13" s="10">
         <v>0</v>
@@ -11812,19 +12828,19 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="4" t="s">
-        <v>298</v>
+        <v>357</v>
       </c>
       <c r="B14" s="4">
         <v>2022</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F14" s="10">
         <v>0</v>
@@ -11835,19 +12851,19 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="4" t="s">
-        <v>299</v>
+        <v>358</v>
       </c>
       <c r="B15" s="4">
         <v>2022</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F15" s="10">
         <v>0</v>
@@ -11858,106 +12874,106 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="4" t="s">
-        <v>300</v>
+        <v>359</v>
       </c>
       <c r="B16" s="4">
         <v>2022</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F16" s="10">
         <v>5</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>302</v>
+        <v>361</v>
       </c>
       <c r="H16" s="4" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="4" t="s">
-        <v>304</v>
+        <v>363</v>
       </c>
       <c r="B17" s="4">
         <v>2022</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F17" s="10">
         <v>29</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>305</v>
+        <v>364</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="4" t="s">
-        <v>306</v>
+        <v>365</v>
       </c>
       <c r="B18" s="4">
         <v>2022</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F18" s="10">
         <v>50</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>307</v>
+        <v>366</v>
       </c>
       <c r="H18" s="4" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="4" t="s">
-        <v>308</v>
+        <v>367</v>
       </c>
       <c r="B19" s="4">
         <v>2022</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F19" s="10">
         <v>0</v>
@@ -11968,19 +12984,19 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="4" t="s">
-        <v>309</v>
+        <v>368</v>
       </c>
       <c r="B20" s="4">
         <v>2023</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>310</v>
+        <v>369</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F20" s="10">
         <v>3</v>
@@ -11991,19 +13007,19 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="4" t="s">
-        <v>311</v>
+        <v>370</v>
       </c>
       <c r="B21" s="4">
         <v>2023</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F21" s="10">
         <v>5</v>
@@ -12014,19 +13030,19 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="4" t="s">
-        <v>312</v>
+        <v>371</v>
       </c>
       <c r="B22" s="4">
         <v>2023</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F22" s="10">
         <v>3</v>
@@ -12037,19 +13053,19 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="4" t="s">
-        <v>313</v>
+        <v>372</v>
       </c>
       <c r="B23" s="4">
         <v>2023</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F23" s="10">
         <v>3</v>
@@ -12060,19 +13076,19 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="4" t="s">
-        <v>314</v>
+        <v>373</v>
       </c>
       <c r="B24" s="4">
         <v>2023</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F24" s="10">
         <v>5</v>
@@ -12083,19 +13099,19 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="4" t="s">
-        <v>315</v>
+        <v>374</v>
       </c>
       <c r="B25" s="4">
         <v>2023</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F25" s="10">
         <v>1</v>
@@ -12106,164 +13122,164 @@
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="4" t="s">
-        <v>316</v>
+        <v>375</v>
       </c>
       <c r="B26" s="4">
         <v>2023</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F26" s="10">
         <v>50</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>317</v>
+        <v>376</v>
       </c>
       <c r="H26" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>318</v>
+        <v>377</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="4" t="s">
-        <v>319</v>
+        <v>378</v>
       </c>
       <c r="B27" s="4">
         <v>2024</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F27" s="10">
         <v>58</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>320</v>
+        <v>379</v>
       </c>
       <c r="H27" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="4" t="s">
-        <v>321</v>
+        <v>380</v>
       </c>
       <c r="B28" s="4">
         <v>2024</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F28" s="10">
         <v>43</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>322</v>
+        <v>381</v>
       </c>
       <c r="H28" s="4" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="4" t="s">
-        <v>323</v>
+        <v>382</v>
       </c>
       <c r="B29" s="4">
         <v>2024</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F29" s="10">
         <v>13.25</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>324</v>
+        <v>383</v>
       </c>
       <c r="H29" s="4" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="4" t="s">
-        <v>325</v>
+        <v>384</v>
       </c>
       <c r="B30" s="4">
         <v>2024</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F30" s="10">
         <v>8.5</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>326</v>
+        <v>385</v>
       </c>
       <c r="H30" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="4" t="s">
-        <v>327</v>
+        <v>386</v>
       </c>
       <c r="B31" s="4">
         <v>2024</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F31" s="10">
         <v>3</v>
@@ -12274,19 +13290,19 @@
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="4" t="s">
-        <v>328</v>
+        <v>387</v>
       </c>
       <c r="B32" s="4">
         <v>2024</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>329</v>
+        <v>388</v>
       </c>
       <c r="F32" s="10">
         <v>0</v>
@@ -12297,19 +13313,19 @@
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="4" t="s">
-        <v>330</v>
+        <v>389</v>
       </c>
       <c r="B33" s="4">
         <v>2024</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>329</v>
+        <v>388</v>
       </c>
       <c r="F33" s="10">
         <v>0</v>
@@ -12320,19 +13336,19 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="4" t="s">
-        <v>331</v>
+        <v>390</v>
       </c>
       <c r="B34" s="4">
         <v>2024</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>285</v>
+        <v>344</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>329</v>
+        <v>388</v>
       </c>
       <c r="F34" s="10">
         <v>0</v>
@@ -12343,19 +13359,19 @@
     </row>
     <row r="35" spans="1:9">
       <c r="A35" s="4" t="s">
-        <v>332</v>
+        <v>391</v>
       </c>
       <c r="B35" s="4">
         <v>2025</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F35" s="10">
         <v>5</v>
@@ -12366,19 +13382,19 @@
     </row>
     <row r="36" spans="1:9">
       <c r="A36" s="4" t="s">
-        <v>333</v>
+        <v>392</v>
       </c>
       <c r="B36" s="4">
         <v>2025</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F36" s="10">
         <v>0</v>
@@ -12389,19 +13405,19 @@
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="4" t="s">
-        <v>334</v>
+        <v>393</v>
       </c>
       <c r="B37" s="4">
         <v>2025</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F37" s="10">
         <v>0</v>
@@ -12412,19 +13428,19 @@
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="4" t="s">
-        <v>335</v>
+        <v>394</v>
       </c>
       <c r="B38" s="4">
         <v>2025</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>286</v>
+        <v>345</v>
       </c>
       <c r="F38" s="10">
         <v>0</v>
@@ -12435,94 +13451,94 @@
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="4" t="s">
-        <v>336</v>
+        <v>395</v>
       </c>
       <c r="B39" s="4">
         <v>2025</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F39" s="10">
         <v>30</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>337</v>
+        <v>396</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="4" t="s">
-        <v>338</v>
+        <v>397</v>
       </c>
       <c r="B40" s="4">
         <v>2025</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>289</v>
+        <v>348</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F40" s="10">
         <v>30</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>339</v>
+        <v>398</v>
       </c>
       <c r="H40" s="4" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>303</v>
+        <v>362</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" s="4" t="s">
-        <v>340</v>
+        <v>399</v>
       </c>
       <c r="B41" s="4">
         <v>2025</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>341</v>
+        <v>400</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>301</v>
+        <v>360</v>
       </c>
       <c r="F41" s="10">
         <v>80</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>342</v>
+        <v>401</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>343</v>
+        <v>402</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="E42" s="3" t="s">
-        <v>344</v>
+        <v>403</v>
       </c>
       <c r="F42" s="10">
         <f>SUM(F4:F41)</f>
@@ -12531,288 +13547,7 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="2" t="s">
-        <v>345</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <cols>
-    <col min="1" max="1" width="22.7109375" customWidth="1"/>
-    <col min="2" max="2" width="60.7109375" customWidth="1"/>
-    <col min="3" max="3" width="8.7109375" customWidth="1"/>
-    <col min="4" max="6" width="28.7109375" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6">
-      <c r="A1" s="1" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
-      <c r="A3" s="3" t="s">
-        <v>168</v>
-      </c>
-      <c r="B3" s="3" t="s">
-        <v>347</v>
-      </c>
-      <c r="C3" s="3" t="s">
-        <v>76</v>
-      </c>
-      <c r="D3" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>349</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>350</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
-      <c r="A4" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="B4" s="4" t="s">
-        <v>351</v>
-      </c>
-      <c r="C4" s="4">
-        <v>2021</v>
-      </c>
-      <c r="D4" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E4" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
-      <c r="A5" s="4" t="s">
-        <v>172</v>
-      </c>
-      <c r="B5" s="4" t="s">
-        <v>353</v>
-      </c>
-      <c r="C5" s="4">
-        <v>2023</v>
-      </c>
-      <c r="D5" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E5" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="F5" s="4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
-      <c r="A6" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B6" s="4" t="s">
-        <v>354</v>
-      </c>
-      <c r="C6" s="4">
-        <v>2023</v>
-      </c>
-      <c r="D6" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E6" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
-      <c r="A7" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>355</v>
-      </c>
-      <c r="C7" s="4">
-        <v>2025</v>
-      </c>
-      <c r="D7" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6">
-      <c r="A8" s="4" t="s">
-        <v>173</v>
-      </c>
-      <c r="B8" s="4" t="s">
-        <v>356</v>
-      </c>
-      <c r="C8" s="4">
-        <v>2023</v>
-      </c>
-      <c r="D8" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E8" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6">
-      <c r="A9" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B9" s="4" t="s">
-        <v>358</v>
-      </c>
-      <c r="C9" s="4">
-        <v>2024</v>
-      </c>
-      <c r="D9" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E9" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6">
-      <c r="A10" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B10" s="4" t="s">
-        <v>359</v>
-      </c>
-      <c r="C10" s="4">
-        <v>2024</v>
-      </c>
-      <c r="D10" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E10" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F10" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6">
-      <c r="A11" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>360</v>
-      </c>
-      <c r="C11" s="4">
-        <v>2024</v>
-      </c>
-      <c r="D11" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E11" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F11" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6">
-      <c r="A12" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B12" s="4" t="s">
-        <v>361</v>
-      </c>
-      <c r="C12" s="4">
-        <v>2024</v>
-      </c>
-      <c r="D12" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6">
-      <c r="A13" s="4" t="s">
-        <v>174</v>
-      </c>
-      <c r="B13" s="4" t="s">
-        <v>362</v>
-      </c>
-      <c r="C13" s="4">
-        <v>2024</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>169</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>357</v>
-      </c>
-      <c r="F13" s="4" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6">
-      <c r="A14" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B14" s="4" t="s">
-        <v>363</v>
-      </c>
-      <c r="C14" s="4">
-        <v>2025</v>
-      </c>
-      <c r="D14" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E14" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="F14" s="4" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6">
-      <c r="A15" s="4" t="s">
-        <v>175</v>
-      </c>
-      <c r="B15" s="4" t="s">
-        <v>364</v>
-      </c>
-      <c r="C15" s="4">
-        <v>2026</v>
-      </c>
-      <c r="D15" s="4" t="s">
-        <v>170</v>
-      </c>
-      <c r="E15" s="4" t="s">
-        <v>352</v>
-      </c>
-      <c r="F15" s="4" t="s">
-        <v>180</v>
+        <v>404</v>
       </c>
     </row>
   </sheetData>
@@ -12834,12 +13569,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -12849,27 +13584,27 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>61</v>
+        <v>64</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B5" s="7">
         <v>42</v>
@@ -12889,7 +13624,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B6" s="7">
         <v>29</v>
@@ -12909,7 +13644,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B7" s="7">
         <v>10</v>
@@ -12929,7 +13664,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="B8" s="7">
         <v>0</v>
@@ -12949,7 +13684,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>70</v>
+        <v>73</v>
       </c>
       <c r="B9" s="7">
         <v>0</v>
@@ -12969,7 +13704,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B10" s="7">
         <v>6</v>
@@ -12989,7 +13724,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B11" s="7">
         <v>1</v>
@@ -13009,7 +13744,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="B12" s="7">
         <v>6</v>
@@ -13039,6 +13774,287 @@
 
 <file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <dimension ref="A1:F15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="2" max="2" width="60.7109375" customWidth="1"/>
+    <col min="3" max="3" width="8.7109375" customWidth="1"/>
+    <col min="4" max="6" width="28.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6">
+      <c r="A1" s="1" t="s">
+        <v>405</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3" s="3" t="s">
+        <v>171</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>406</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>407</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>408</v>
+      </c>
+      <c r="F3" s="3" t="s">
+        <v>409</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>410</v>
+      </c>
+      <c r="C4" s="4">
+        <v>2021</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5" s="4" t="s">
+        <v>175</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>412</v>
+      </c>
+      <c r="C5" s="4">
+        <v>2023</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B6" s="4" t="s">
+        <v>413</v>
+      </c>
+      <c r="C6" s="4">
+        <v>2023</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" s="4" t="s">
+        <v>414</v>
+      </c>
+      <c r="C7" s="4">
+        <v>2025</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F7" s="4" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>415</v>
+      </c>
+      <c r="C8" s="4">
+        <v>2023</v>
+      </c>
+      <c r="D8" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>417</v>
+      </c>
+      <c r="C9" s="4">
+        <v>2024</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B10" s="4" t="s">
+        <v>418</v>
+      </c>
+      <c r="C10" s="4">
+        <v>2024</v>
+      </c>
+      <c r="D10" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E10" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F10" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B11" s="4" t="s">
+        <v>419</v>
+      </c>
+      <c r="C11" s="4">
+        <v>2024</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E11" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F11" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6">
+      <c r="A12" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>420</v>
+      </c>
+      <c r="C12" s="4">
+        <v>2024</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6">
+      <c r="A13" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>421</v>
+      </c>
+      <c r="C13" s="4">
+        <v>2024</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>416</v>
+      </c>
+      <c r="F13" s="4" t="s">
+        <v>182</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6">
+      <c r="A14" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>422</v>
+      </c>
+      <c r="C14" s="4">
+        <v>2025</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F14" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6">
+      <c r="A15" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>423</v>
+      </c>
+      <c r="C15" s="4">
+        <v>2026</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>411</v>
+      </c>
+      <c r="F15" s="4" t="s">
+        <v>183</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:D19"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -13050,245 +14066,245 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>365</v>
+        <v>424</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="3" t="s">
-        <v>366</v>
+        <v>204</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>367</v>
+        <v>425</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>368</v>
+        <v>426</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>369</v>
+        <v>427</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>370</v>
+        <v>428</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>371</v>
+        <v>429</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="4" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>430</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>120</v>
       </c>
-      <c r="B5" s="4" t="s">
-        <v>372</v>
-      </c>
-      <c r="C5" s="4" t="s">
-        <v>117</v>
-      </c>
       <c r="D5" s="4" t="s">
-        <v>373</v>
+        <v>431</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>374</v>
+        <v>432</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>375</v>
+        <v>433</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>376</v>
+        <v>434</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>377</v>
+        <v>435</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>378</v>
+        <v>436</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>379</v>
+        <v>437</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="4" t="s">
+        <v>124</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>438</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>121</v>
       </c>
-      <c r="B9" s="4" t="s">
-        <v>380</v>
-      </c>
-      <c r="C9" s="4" t="s">
-        <v>118</v>
-      </c>
       <c r="D9" s="4" t="s">
-        <v>381</v>
+        <v>439</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>382</v>
+        <v>440</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>383</v>
+        <v>441</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>384</v>
+        <v>442</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>385</v>
+        <v>443</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>386</v>
+        <v>444</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>385</v>
+        <v>443</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>387</v>
+        <v>445</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>385</v>
+        <v>443</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>388</v>
+        <v>446</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>389</v>
+        <v>447</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>390</v>
+        <v>448</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>391</v>
+        <v>449</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>392</v>
+        <v>450</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>393</v>
+        <v>451</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>394</v>
+        <v>452</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>395</v>
+        <v>453</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>396</v>
+        <v>454</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>397</v>
+        <v>455</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>398</v>
+        <v>456</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>399</v>
+        <v>457</v>
       </c>
     </row>
   </sheetData>
@@ -13310,12 +14326,12 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:9" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -13328,36 +14344,36 @@
     </row>
     <row r="4" spans="1:9" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>78</v>
+        <v>81</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B5" s="7">
         <v>17</v>
@@ -13386,7 +14402,7 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B6" s="7">
         <v>42</v>
@@ -13415,7 +14431,7 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" s="7">
         <v>50</v>
@@ -13444,7 +14460,7 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="7">
         <v>72</v>
@@ -13473,7 +14489,7 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B9" s="7">
         <v>109</v>
@@ -13524,12 +14540,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -13539,21 +14555,21 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B5" s="7">
         <v>23</v>
@@ -13567,7 +14583,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B6" s="7">
         <v>55</v>
@@ -13581,7 +14597,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" s="7">
         <v>61</v>
@@ -13595,7 +14611,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="7">
         <v>105</v>
@@ -13609,7 +14625,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B9" s="7">
         <v>161</v>
@@ -13645,12 +14661,12 @@
   <sheetData>
     <row r="1" spans="1:7">
       <c r="A1" s="1" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
     </row>
     <row r="2" spans="1:7" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -13661,30 +14677,30 @@
     </row>
     <row r="4" spans="1:7" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>98</v>
+        <v>101</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>99</v>
+        <v>102</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>100</v>
+        <v>103</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
     </row>
     <row r="5" spans="1:7">
       <c r="A5" s="4" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="B5" s="7">
         <v>0</v>
@@ -13707,7 +14723,7 @@
     </row>
     <row r="6" spans="1:7">
       <c r="A6" s="4" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="B6" s="7">
         <v>1</v>
@@ -13730,7 +14746,7 @@
     </row>
     <row r="7" spans="1:7">
       <c r="A7" s="4" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B7" s="7">
         <v>1</v>
@@ -13753,7 +14769,7 @@
     </row>
     <row r="8" spans="1:7">
       <c r="A8" s="4" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="B8" s="7">
         <v>9</v>
@@ -13776,7 +14792,7 @@
     </row>
     <row r="9" spans="1:7">
       <c r="A9" s="4" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="B9" s="7">
         <v>8</v>
@@ -13821,12 +14837,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -13836,21 +14852,21 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>60</v>
+        <v>63</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="B5" s="7">
         <v>29</v>
@@ -13864,7 +14880,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="B6" s="7">
         <v>47</v>
@@ -13878,7 +14894,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="B7" s="7">
         <v>70</v>
@@ -13892,7 +14908,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="B8" s="7">
         <v>6</v>
@@ -13906,7 +14922,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B9" s="7">
         <v>12</v>
@@ -13942,12 +14958,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -13957,15 +14973,15 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="B5" s="7">
         <v>88</v>
@@ -13973,7 +14989,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="B6" s="7">
         <v>159</v>
@@ -14003,12 +15019,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -14018,21 +15034,21 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="B5" s="7">
         <v>1</v>
@@ -14046,7 +15062,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B6" s="7">
         <v>1</v>
@@ -14060,7 +15076,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B7" s="7">
         <v>3</v>
@@ -14074,7 +15090,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="B8" s="7">
         <v>0</v>
@@ -14110,12 +15126,12 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
       <c r="A2" s="6" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -14125,27 +15141,27 @@
     </row>
     <row r="4" spans="1:6" ht="45" customHeight="1">
       <c r="A4" s="3" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
     </row>
     <row r="5" spans="1:6">
       <c r="A5" s="4" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="B5" s="7">
         <v>0</v>
@@ -14165,7 +15181,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="4" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="B6" s="7">
         <v>30</v>
@@ -14185,7 +15201,7 @@
     </row>
     <row r="7" spans="1:6">
       <c r="A7" s="4" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="B7" s="7">
         <v>60</v>
@@ -14205,7 +15221,7 @@
     </row>
     <row r="8" spans="1:6">
       <c r="A8" s="4" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B8" s="7">
         <v>90</v>
@@ -14225,7 +15241,7 @@
     </row>
     <row r="9" spans="1:6">
       <c r="A9" s="4" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="B9" s="7">
         <v>100</v>
@@ -14245,7 +15261,7 @@
     </row>
     <row r="10" spans="1:6">
       <c r="A10" s="4" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B10" s="7">
         <v>100</v>
@@ -14265,7 +15281,7 @@
     </row>
     <row r="11" spans="1:6">
       <c r="A11" s="4" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B11" s="7">
         <v>100</v>
@@ -14285,7 +15301,7 @@
     </row>
     <row r="12" spans="1:6">
       <c r="A12" s="4" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="B12" s="7">
         <v>100</v>

</xml_diff>

<commit_message>
Chuyển nội dung Thông tư 83/2026 từ Chương 2 sang mục Thời cơ và thách thức của Chương 3
Thông tư có hiệu lực từ 15/11/2026, chưa áp dụng cho giai đoạn đánh giá thực trạng.
Chương 2 bỏ Mục 2.1.3 và các câu liên quan, số bảng tự đánh lại; Chương 3 thêm Mục 3.1.2 Thời cơ và thách thức
ở chế độ theo dõi thay đổi, Mục 3.1.2 cũ thành 3.1.3.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThGArqDrUUsqC1zG1BQvVL
</commit_message>
<xml_diff>
--- a/Du_lieu_bieu_do_Chuong_2.xlsx
+++ b/Du_lieu_bieu_do_Chuong_2.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="640" uniqueCount="412">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="636" uniqueCount="409">
   <si>
     <t>DỮ LIỆU VÀ BIỂU ĐỒ CHƯƠNG 2 - THỰC TRẠNG QUẢN LÝ QUYỀN SỞ HỮU TRÍ TUỆ TẠI TRƯỜNG ĐẠI HỌC THÀNH ĐÔ</t>
   </si>
@@ -335,39 +335,39 @@
     <t>Hình 2.6. Tài sản trí tuệ của Nhà trường theo loại hình và tình trạng pháp lý</t>
   </si>
   <si>
+    <t>Nguồn: Nhóm nghiên cứu tổng hợp từ Bảng 2.6.</t>
+  </si>
+  <si>
+    <t>Loại hình</t>
+  </si>
+  <si>
+    <t>Đã cấp văn bằng</t>
+  </si>
+  <si>
+    <t>Đang xử lý</t>
+  </si>
+  <si>
+    <t>Trong đó đồng sở hữu với doanh nghiệp</t>
+  </si>
+  <si>
+    <t>Quyền tác giả</t>
+  </si>
+  <si>
+    <t>Nhãn hiệu</t>
+  </si>
+  <si>
+    <t>Kiểu dáng công nghiệp</t>
+  </si>
+  <si>
+    <t>Sáng chế</t>
+  </si>
+  <si>
+    <t>Hình 2.7. Sản phẩm đề tài cấp cơ sở đủ điều kiện xác lập quyền theo nhóm quyền có thể xác lập</t>
+  </si>
+  <si>
     <t>Nguồn: Nhóm nghiên cứu tổng hợp từ Bảng 2.7.</t>
   </si>
   <si>
-    <t>Loại hình</t>
-  </si>
-  <si>
-    <t>Đã cấp văn bằng</t>
-  </si>
-  <si>
-    <t>Đang xử lý</t>
-  </si>
-  <si>
-    <t>Trong đó đồng sở hữu với doanh nghiệp</t>
-  </si>
-  <si>
-    <t>Quyền tác giả</t>
-  </si>
-  <si>
-    <t>Nhãn hiệu</t>
-  </si>
-  <si>
-    <t>Kiểu dáng công nghiệp</t>
-  </si>
-  <si>
-    <t>Sáng chế</t>
-  </si>
-  <si>
-    <t>Hình 2.7. Sản phẩm đề tài cấp cơ sở đủ điều kiện xác lập quyền theo nhóm quyền có thể xác lập</t>
-  </si>
-  <si>
-    <t>Nguồn: Nhóm nghiên cứu tổng hợp từ Bảng 2.8.</t>
-  </si>
-  <si>
     <t>Nhóm quyền có thể xác lập</t>
   </si>
   <si>
@@ -386,7 +386,7 @@
     <t>Hình 2.8. Chuỗi chuyển hóa từ đề tài cấp cơ sở sang đơn đăng ký sở hữu công nghiệp</t>
   </si>
   <si>
-    <t>Nguồn: Nhóm nghiên cứu tính toán từ danh mục đề tài cấp cơ sở và Bảng 2.8.</t>
+    <t>Nguồn: Nhóm nghiên cứu tính toán từ danh mục đề tài cấp cơ sở và Bảng 2.7.</t>
   </si>
   <si>
     <t>Bậc chuyển hóa</t>
@@ -503,25 +503,16 @@
     <t>Xác nhận của chủ nhiệm đề tài</t>
   </si>
   <si>
-    <t>Mục 2.1.3 mới</t>
+    <t>Thông tư 83/2026/TT-BGDĐT về Chuẩn cơ sở giáo dục đại học</t>
   </si>
   <si>
     <t>Chưa có</t>
   </si>
   <si>
-    <t>Đối chiếu Thông tư 83/2026/TT-BGDĐT với Thông tư 01/2024/TT-BGDĐT; ước tính chỉ số 6.2 năm 2025</t>
-  </si>
-  <si>
-    <t>VBPL/01_2024_TT-BGDDT; 83_2026_TT-BGDDT_727285.docx, Điều 6, Phụ lục I Bảng 1, Phụ lục II mục 6.2</t>
-  </si>
-  <si>
-    <t>Giảng viên quy đổi</t>
-  </si>
-  <si>
-    <t>83 x 1,0 + 58 x 0,75 + 3 x 0,5 = 128,0</t>
-  </si>
-  <si>
-    <t>2026 DS.xlsx, cột học hàm, học vị của 145 giảng viên; 1 giảng viên trình độ trung cấp không tính</t>
+    <t>Không đưa vào Chương 2 vì Thông tư có hiệu lực từ ngày 15 tháng 11 năm 2026, chưa áp dụng cho giai đoạn đánh giá; được đưa vào Mục 3.1.2 Thời cơ và thách thức của Chương 3</t>
+  </si>
+  <si>
+    <t>Ý kiến của chủ nhiệm đề tài</t>
   </si>
   <si>
     <t>Ngân sách Quỹ Ngô Xuân Độ</t>
@@ -7156,7 +7147,7 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D39"/>
+  <dimension ref="A1:D38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="32.7109375" customWidth="1"/>
@@ -7244,13 +7235,13 @@
         <v>162</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>159</v>
+        <v>163</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>164</v>
+        <v>157</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -7264,161 +7255,161 @@
         <v>167</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>157</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="4" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="4" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="4" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="4" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="4" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="4" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="4" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="4" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>211</v>
+        <v>172</v>
       </c>
     </row>
     <row r="21" spans="1:4">
@@ -7432,96 +7423,96 @@
         <v>214</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>175</v>
+        <v>215</v>
       </c>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="4" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="4" t="s">
-        <v>219</v>
+        <v>220</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>220</v>
+        <v>51</v>
       </c>
       <c r="C23" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="D23" s="4" t="s">
         <v>221</v>
-      </c>
-      <c r="D23" s="4" t="s">
-        <v>222</v>
       </c>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="4" t="s">
+        <v>222</v>
+      </c>
+      <c r="B24" s="4" t="s">
         <v>223</v>
       </c>
-      <c r="B24" s="4" t="s">
-        <v>51</v>
-      </c>
       <c r="C24" s="4" t="s">
-        <v>52</v>
+        <v>224</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>224</v>
+        <v>225</v>
       </c>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="4" t="s">
-        <v>225</v>
+        <v>226</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="4" t="s">
-        <v>229</v>
+        <v>230</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>230</v>
+        <v>231</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="4" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>235</v>
+        <v>236</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="4" t="s">
-        <v>237</v>
+        <v>154</v>
       </c>
       <c r="B28" s="4" t="s">
         <v>238</v>
@@ -7535,95 +7526,93 @@
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="4" t="s">
-        <v>154</v>
+        <v>241</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>241</v>
+        <v>242</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>242</v>
+        <v>243</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>243</v>
+        <v>244</v>
       </c>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="4" t="s">
-        <v>244</v>
+        <v>245</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>246</v>
+        <v>247</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>247</v>
+        <v>248</v>
       </c>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="4" t="s">
-        <v>248</v>
+        <v>249</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>249</v>
+        <v>250</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>250</v>
+        <v>251</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>251</v>
+        <v>252</v>
       </c>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="4" t="s">
-        <v>252</v>
+        <v>253</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>253</v>
+        <v>254</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>254</v>
+        <v>255</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>255</v>
+        <v>256</v>
       </c>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="4" t="s">
-        <v>256</v>
+        <v>257</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>257</v>
+        <v>258</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>258</v>
+        <v>259</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>259</v>
+        <v>260</v>
       </c>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="4" t="s">
-        <v>260</v>
+        <v>261</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>261</v>
+        <v>262</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>263</v>
+        <v>264</v>
       </c>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="4" t="s">
-        <v>264</v>
-      </c>
-      <c r="B35" s="4" t="s">
         <v>265</v>
       </c>
+      <c r="B35" s="4"/>
       <c r="C35" s="4" t="s">
         <v>266</v>
       </c>
@@ -7635,50 +7624,38 @@
       <c r="A36" s="4" t="s">
         <v>268</v>
       </c>
-      <c r="B36" s="4"/>
+      <c r="B36" s="4" t="s">
+        <v>269</v>
+      </c>
       <c r="C36" s="4" t="s">
-        <v>269</v>
+        <v>270</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="4" t="s">
-        <v>271</v>
-      </c>
-      <c r="B37" s="4" t="s">
         <v>272</v>
       </c>
+      <c r="B37" s="4"/>
       <c r="C37" s="4" t="s">
         <v>273</v>
       </c>
-      <c r="D37" s="4" t="s">
-        <v>274</v>
-      </c>
+      <c r="D37" s="4"/>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="4" t="s">
+        <v>274</v>
+      </c>
+      <c r="B38" s="4" t="s">
         <v>275</v>
       </c>
-      <c r="B38" s="4"/>
       <c r="C38" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="D38" s="4"/>
-    </row>
-    <row r="39" spans="1:4">
-      <c r="A39" s="4" t="s">
+      <c r="D38" s="4" t="s">
         <v>277</v>
-      </c>
-      <c r="B39" s="4" t="s">
-        <v>278</v>
-      </c>
-      <c r="C39" s="4" t="s">
-        <v>279</v>
-      </c>
-      <c r="D39" s="4" t="s">
-        <v>280</v>
       </c>
     </row>
   </sheetData>
@@ -7699,53 +7676,53 @@
   <sheetData>
     <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>42</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>280</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>281</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>282</v>
+      </c>
+      <c r="F3" s="3" t="s">
         <v>283</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>284</v>
-      </c>
-      <c r="E3" s="3" t="s">
-        <v>285</v>
-      </c>
-      <c r="F3" s="3" t="s">
-        <v>286</v>
-      </c>
-      <c r="G3" s="3" t="s">
-        <v>287</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>113</v>
       </c>
       <c r="I3" s="3" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
     </row>
     <row r="4" spans="1:9">
       <c r="A4" s="4" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="B4" s="4">
         <v>2021</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F4" s="8">
         <v>0</v>
@@ -7756,19 +7733,19 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" s="4" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="B5" s="4">
         <v>2021</v>
       </c>
       <c r="C5" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F5" s="8">
         <v>0</v>
@@ -7779,19 +7756,19 @@
     </row>
     <row r="6" spans="1:9">
       <c r="A6" s="4" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="B6" s="4">
         <v>2021</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F6" s="8">
         <v>0</v>
@@ -7802,19 +7779,19 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" s="4" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="B7" s="4">
         <v>2021</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F7" s="8">
         <v>0</v>
@@ -7825,19 +7802,19 @@
     </row>
     <row r="8" spans="1:9">
       <c r="A8" s="4" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="B8" s="4">
         <v>2021</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F8" s="8">
         <v>0</v>
@@ -7848,19 +7825,19 @@
     </row>
     <row r="9" spans="1:9">
       <c r="A9" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B9" s="4">
         <v>2021</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F9" s="8">
         <v>0</v>
@@ -7871,19 +7848,19 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" s="4" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B10" s="4">
         <v>2022</v>
       </c>
       <c r="C10" s="4" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F10" s="8">
         <v>0</v>
@@ -7894,19 +7871,19 @@
     </row>
     <row r="11" spans="1:9">
       <c r="A11" s="4" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="B11" s="4">
         <v>2022</v>
       </c>
       <c r="C11" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F11" s="8">
         <v>0</v>
@@ -7917,19 +7894,19 @@
     </row>
     <row r="12" spans="1:9">
       <c r="A12" s="4" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="B12" s="4">
         <v>2022</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F12" s="8">
         <v>0</v>
@@ -7940,19 +7917,19 @@
     </row>
     <row r="13" spans="1:9">
       <c r="A13" s="4" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="B13" s="4">
         <v>2022</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F13" s="8">
         <v>0</v>
@@ -7963,19 +7940,19 @@
     </row>
     <row r="14" spans="1:9">
       <c r="A14" s="4" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="B14" s="4">
         <v>2022</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F14" s="8">
         <v>0</v>
@@ -7986,19 +7963,19 @@
     </row>
     <row r="15" spans="1:9">
       <c r="A15" s="4" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="B15" s="4">
         <v>2022</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F15" s="8">
         <v>0</v>
@@ -8009,106 +7986,106 @@
     </row>
     <row r="16" spans="1:9">
       <c r="A16" s="4" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="B16" s="4">
         <v>2022</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F16" s="8">
         <v>5</v>
       </c>
       <c r="G16" s="4" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>117</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" s="4" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="B17" s="4">
         <v>2022</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F17" s="8">
         <v>29</v>
       </c>
       <c r="G17" s="4" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>115</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" s="4" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="B18" s="4">
         <v>2022</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F18" s="8">
         <v>50</v>
       </c>
       <c r="G18" s="4" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>116</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" s="4" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="B19" s="4">
         <v>2022</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F19" s="8">
         <v>0</v>
@@ -8119,19 +8096,19 @@
     </row>
     <row r="20" spans="1:9">
       <c r="A20" s="4" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="B20" s="4">
         <v>2023</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>319</v>
+        <v>316</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F20" s="8">
         <v>3</v>
@@ -8142,19 +8119,19 @@
     </row>
     <row r="21" spans="1:9">
       <c r="A21" s="4" t="s">
-        <v>320</v>
+        <v>317</v>
       </c>
       <c r="B21" s="4">
         <v>2023</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F21" s="8">
         <v>5</v>
@@ -8165,19 +8142,19 @@
     </row>
     <row r="22" spans="1:9">
       <c r="A22" s="4" t="s">
-        <v>321</v>
+        <v>318</v>
       </c>
       <c r="B22" s="4">
         <v>2023</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F22" s="8">
         <v>3</v>
@@ -8188,19 +8165,19 @@
     </row>
     <row r="23" spans="1:9">
       <c r="A23" s="4" t="s">
-        <v>322</v>
+        <v>319</v>
       </c>
       <c r="B23" s="4">
         <v>2023</v>
       </c>
       <c r="C23" s="4" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F23" s="8">
         <v>3</v>
@@ -8211,19 +8188,19 @@
     </row>
     <row r="24" spans="1:9">
       <c r="A24" s="4" t="s">
-        <v>323</v>
+        <v>320</v>
       </c>
       <c r="B24" s="4">
         <v>2023</v>
       </c>
       <c r="C24" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F24" s="8">
         <v>5</v>
@@ -8234,19 +8211,19 @@
     </row>
     <row r="25" spans="1:9">
       <c r="A25" s="4" t="s">
-        <v>324</v>
+        <v>321</v>
       </c>
       <c r="B25" s="4">
         <v>2023</v>
       </c>
       <c r="C25" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F25" s="8">
         <v>1</v>
@@ -8257,164 +8234,164 @@
     </row>
     <row r="26" spans="1:9">
       <c r="A26" s="4" t="s">
-        <v>325</v>
+        <v>322</v>
       </c>
       <c r="B26" s="4">
         <v>2023</v>
       </c>
       <c r="C26" s="4" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F26" s="8">
         <v>50</v>
       </c>
       <c r="G26" s="4" t="s">
-        <v>327</v>
+        <v>324</v>
       </c>
       <c r="H26" s="4" t="s">
         <v>85</v>
       </c>
       <c r="I26" s="4" t="s">
-        <v>328</v>
+        <v>325</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" s="4" t="s">
-        <v>329</v>
+        <v>326</v>
       </c>
       <c r="B27" s="4">
         <v>2024</v>
       </c>
       <c r="C27" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F27" s="8">
         <v>58</v>
       </c>
       <c r="G27" s="4" t="s">
-        <v>330</v>
+        <v>327</v>
       </c>
       <c r="H27" s="4" t="s">
         <v>85</v>
       </c>
       <c r="I27" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" s="4" t="s">
-        <v>331</v>
+        <v>328</v>
       </c>
       <c r="B28" s="4">
         <v>2024</v>
       </c>
       <c r="C28" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D28" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F28" s="8">
         <v>43</v>
       </c>
       <c r="G28" s="4" t="s">
-        <v>332</v>
+        <v>329</v>
       </c>
       <c r="H28" s="4" t="s">
         <v>116</v>
       </c>
       <c r="I28" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" s="4" t="s">
-        <v>333</v>
+        <v>330</v>
       </c>
       <c r="B29" s="4">
         <v>2024</v>
       </c>
       <c r="C29" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F29" s="8">
         <v>13.25</v>
       </c>
       <c r="G29" s="4" t="s">
-        <v>334</v>
+        <v>331</v>
       </c>
       <c r="H29" s="4" t="s">
         <v>115</v>
       </c>
       <c r="I29" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" s="4" t="s">
-        <v>335</v>
+        <v>332</v>
       </c>
       <c r="B30" s="4">
         <v>2024</v>
       </c>
       <c r="C30" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F30" s="8">
         <v>8.5</v>
       </c>
       <c r="G30" s="4" t="s">
-        <v>336</v>
+        <v>333</v>
       </c>
       <c r="H30" s="4" t="s">
         <v>85</v>
       </c>
       <c r="I30" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" s="4" t="s">
-        <v>337</v>
+        <v>334</v>
       </c>
       <c r="B31" s="4">
         <v>2024</v>
       </c>
       <c r="C31" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F31" s="8">
         <v>3</v>
@@ -8425,19 +8402,19 @@
     </row>
     <row r="32" spans="1:9">
       <c r="A32" s="4" t="s">
-        <v>338</v>
+        <v>335</v>
       </c>
       <c r="B32" s="4">
         <v>2024</v>
       </c>
       <c r="C32" s="4" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D32" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F32" s="8">
         <v>0</v>
@@ -8448,19 +8425,19 @@
     </row>
     <row r="33" spans="1:9">
       <c r="A33" s="4" t="s">
-        <v>340</v>
+        <v>337</v>
       </c>
       <c r="B33" s="4">
         <v>2024</v>
       </c>
       <c r="C33" s="4" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="D33" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F33" s="8">
         <v>0</v>
@@ -8471,19 +8448,19 @@
     </row>
     <row r="34" spans="1:9">
       <c r="A34" s="4" t="s">
-        <v>341</v>
+        <v>338</v>
       </c>
       <c r="B34" s="4">
         <v>2024</v>
       </c>
       <c r="C34" s="4" t="s">
-        <v>326</v>
+        <v>323</v>
       </c>
       <c r="D34" s="4" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>339</v>
+        <v>336</v>
       </c>
       <c r="F34" s="8">
         <v>0</v>
@@ -8494,19 +8471,19 @@
     </row>
     <row r="35" spans="1:9">
       <c r="A35" s="4" t="s">
-        <v>342</v>
+        <v>339</v>
       </c>
       <c r="B35" s="4">
         <v>2025</v>
       </c>
       <c r="C35" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D35" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F35" s="8">
         <v>5</v>
@@ -8517,19 +8494,19 @@
     </row>
     <row r="36" spans="1:9">
       <c r="A36" s="4" t="s">
-        <v>343</v>
+        <v>340</v>
       </c>
       <c r="B36" s="4">
         <v>2025</v>
       </c>
       <c r="C36" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D36" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F36" s="8">
         <v>0</v>
@@ -8540,19 +8517,19 @@
     </row>
     <row r="37" spans="1:9">
       <c r="A37" s="4" t="s">
-        <v>344</v>
+        <v>341</v>
       </c>
       <c r="B37" s="4">
         <v>2025</v>
       </c>
       <c r="C37" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F37" s="8">
         <v>0</v>
@@ -8563,19 +8540,19 @@
     </row>
     <row r="38" spans="1:9">
       <c r="A38" s="4" t="s">
-        <v>345</v>
+        <v>342</v>
       </c>
       <c r="B38" s="4">
         <v>2025</v>
       </c>
       <c r="C38" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D38" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="F38" s="8">
         <v>0</v>
@@ -8586,94 +8563,94 @@
     </row>
     <row r="39" spans="1:9">
       <c r="A39" s="4" t="s">
-        <v>346</v>
+        <v>343</v>
       </c>
       <c r="B39" s="4">
         <v>2025</v>
       </c>
       <c r="C39" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F39" s="8">
         <v>30</v>
       </c>
       <c r="G39" s="4" t="s">
-        <v>347</v>
+        <v>344</v>
       </c>
       <c r="H39" s="4" t="s">
         <v>85</v>
       </c>
       <c r="I39" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" s="4" t="s">
-        <v>348</v>
+        <v>345</v>
       </c>
       <c r="B40" s="4">
         <v>2025</v>
       </c>
       <c r="C40" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D40" s="4" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="E40" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F40" s="8">
         <v>30</v>
       </c>
       <c r="G40" s="4" t="s">
-        <v>349</v>
+        <v>346</v>
       </c>
       <c r="H40" s="4" t="s">
         <v>85</v>
       </c>
       <c r="I40" s="4" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" s="4" t="s">
-        <v>350</v>
+        <v>347</v>
       </c>
       <c r="B41" s="4">
         <v>2025</v>
       </c>
       <c r="C41" s="4" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D41" s="4" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="F41" s="8">
         <v>80</v>
       </c>
       <c r="G41" s="4" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
       <c r="H41" s="4" t="s">
         <v>110</v>
       </c>
       <c r="I41" s="4" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="E42" s="3" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="F42" s="8">
         <f>SUM(F4:F41)</f>
@@ -8682,7 +8659,7 @@
     </row>
     <row r="44" spans="1:9">
       <c r="A44" s="2" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
     </row>
   </sheetData>
@@ -8703,7 +8680,7 @@
   <sheetData>
     <row r="1" spans="1:6">
       <c r="A1" s="1" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
     </row>
     <row r="3" spans="1:6">
@@ -8711,19 +8688,19 @@
         <v>103</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
       <c r="C3" s="3" t="s">
         <v>42</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
       <c r="E3" s="3" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -8731,7 +8708,7 @@
         <v>107</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
       <c r="C4" s="4">
         <v>2021</v>
@@ -8740,10 +8717,10 @@
         <v>104</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -8751,7 +8728,7 @@
         <v>107</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="C5" s="4">
         <v>2023</v>
@@ -8760,10 +8737,10 @@
         <v>104</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F5" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -8771,7 +8748,7 @@
         <v>108</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="C6" s="4">
         <v>2023</v>
@@ -8780,10 +8757,10 @@
         <v>104</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F6" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -8791,7 +8768,7 @@
         <v>108</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="C7" s="4">
         <v>2025</v>
@@ -8800,10 +8777,10 @@
         <v>104</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F7" s="4" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -8811,7 +8788,7 @@
         <v>108</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="C8" s="4">
         <v>2023</v>
@@ -8820,10 +8797,10 @@
         <v>105</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F8" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -8831,7 +8808,7 @@
         <v>109</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="C9" s="4">
         <v>2024</v>
@@ -8840,10 +8817,10 @@
         <v>104</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F9" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -8851,7 +8828,7 @@
         <v>109</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="C10" s="4">
         <v>2024</v>
@@ -8860,10 +8837,10 @@
         <v>104</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -8871,7 +8848,7 @@
         <v>109</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
       <c r="C11" s="4">
         <v>2024</v>
@@ -8880,10 +8857,10 @@
         <v>104</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F11" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -8891,7 +8868,7 @@
         <v>109</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="C12" s="4">
         <v>2024</v>
@@ -8900,10 +8877,10 @@
         <v>104</v>
       </c>
       <c r="E12" s="4" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F12" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -8911,7 +8888,7 @@
         <v>109</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="C13" s="4">
         <v>2024</v>
@@ -8920,10 +8897,10 @@
         <v>104</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -8931,7 +8908,7 @@
         <v>110</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="C14" s="4">
         <v>2025</v>
@@ -8940,10 +8917,10 @@
         <v>105</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -8951,7 +8928,7 @@
         <v>110</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
       <c r="C15" s="4">
         <v>2026</v>
@@ -8960,10 +8937,10 @@
         <v>105</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
     </row>
   </sheetData>
@@ -8984,7 +8961,7 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="1" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
     </row>
     <row r="3" spans="1:4">
@@ -8992,13 +8969,13 @@
         <v>129</v>
       </c>
       <c r="B3" s="3" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
     </row>
     <row r="4" spans="1:4">
@@ -9006,13 +8983,13 @@
         <v>97</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C4" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
     </row>
     <row r="5" spans="1:4">
@@ -9020,13 +8997,13 @@
         <v>97</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="C5" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
     </row>
     <row r="6" spans="1:4">
@@ -9034,13 +9011,13 @@
         <v>97</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="C6" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
     </row>
     <row r="7" spans="1:4">
@@ -9048,13 +9025,13 @@
         <v>98</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="C7" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D7" s="4" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
     </row>
     <row r="8" spans="1:4">
@@ -9062,13 +9039,13 @@
         <v>98</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
     </row>
     <row r="9" spans="1:4">
@@ -9076,13 +9053,13 @@
         <v>98</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D9" s="4" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
     </row>
     <row r="10" spans="1:4">
@@ -9090,13 +9067,13 @@
         <v>98</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
     </row>
     <row r="11" spans="1:4">
@@ -9104,13 +9081,13 @@
         <v>99</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="12" spans="1:4">
@@ -9118,13 +9095,13 @@
         <v>99</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="13" spans="1:4">
@@ -9132,13 +9109,13 @@
         <v>99</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>94</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
     </row>
     <row r="14" spans="1:4">
@@ -9146,13 +9123,13 @@
         <v>99</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="C14" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
     </row>
     <row r="15" spans="1:4">
@@ -9160,13 +9137,13 @@
         <v>100</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="C15" s="4" t="s">
         <v>95</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
     </row>
     <row r="16" spans="1:4">
@@ -9174,13 +9151,13 @@
         <v>100</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="C16" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
     </row>
     <row r="17" spans="1:4">
@@ -9188,13 +9165,13 @@
         <v>100</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="C17" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
     </row>
     <row r="18" spans="1:4">
@@ -9202,13 +9179,13 @@
         <v>100</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
     </row>
     <row r="19" spans="1:4">
@@ -9216,13 +9193,13 @@
         <v>100</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>96</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
     </row>
   </sheetData>

</xml_diff>